<commit_message>
B2B rooms/rooming list fixes ?
</commit_message>
<xml_diff>
--- a/app/templates/report/rooming.xlsx
+++ b/app/templates/report/rooming.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\ciber\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD2FB1B9-CCB7-49E1-855D-71915E9B3A8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55ECDFFE-9A34-44C0-989E-BD04BE847C50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rooming" sheetId="1" r:id="rId1"/>
-    <sheet name="Rooms" sheetId="8" state="hidden" r:id="rId2"/>
-    <sheet name="Idtype" sheetId="4" state="hidden" r:id="rId3"/>
-    <sheet name="Gender" sheetId="6" state="hidden" r:id="rId4"/>
-    <sheet name="Country" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet name="Language" sheetId="7" state="hidden" r:id="rId6"/>
+    <sheet name="_Rooms" sheetId="8" state="hidden" r:id="rId2"/>
+    <sheet name="_Idtype" sheetId="4" state="hidden" r:id="rId3"/>
+    <sheet name="_Gender" sheetId="6" state="hidden" r:id="rId4"/>
+    <sheet name="_Country" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="_Language" sheetId="7" state="hidden" r:id="rId6"/>
+    <sheet name="_Check" sheetId="9" state="hidden" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="49">
   <si>
     <t>ROOMING LIST</t>
   </si>
@@ -163,7 +164,30 @@
     <t>Code</t>
   </si>
   <si>
-    <t>Room.Code</t>
+    <t>Check_in_ok</t>
+  </si>
+  <si>
+    <t>Revisiòn
+Ok</t>
+  </si>
+  <si>
+    <t>Revision_ok</t>
+  </si>
+  <si>
+    <t>Limpieza Fcturada</t>
+  </si>
+  <si>
+    <t>Cleaning_billed</t>
+  </si>
+  <si>
+    <t>Check</t>
+  </si>
+  <si>
+    <t>Check-in
+Ok</t>
+  </si>
+  <si>
+    <t>Resource.Code</t>
   </si>
 </sst>
 </file>
@@ -457,7 +481,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -564,6 +588,14 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -571,16 +603,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <border>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <border>
         <top style="thin">
@@ -1022,33 +1045,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:U5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.7109375" style="5" customWidth="1"/>
     <col min="2" max="2" width="10.140625" style="11" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.5703125" style="11" customWidth="1"/>
     <col min="4" max="4" width="9.140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.42578125" style="12" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.5703125" style="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28.7109375" style="12" customWidth="1"/>
-    <col min="8" max="8" width="15.28515625" style="12" customWidth="1"/>
-    <col min="9" max="9" width="28.7109375" style="12" customWidth="1"/>
-    <col min="10" max="10" width="15.5703125" style="12" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.7109375" style="12" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6" style="12" bestFit="1" customWidth="1"/>
-    <col min="13" max="18" width="17.7109375" style="12" customWidth="1"/>
-    <col min="19" max="246" width="9.140625" style="5" customWidth="1"/>
-    <col min="247" max="247" width="11.42578125" style="5" customWidth="1"/>
-    <col min="248" max="16384" width="11.42578125" style="5"/>
+    <col min="5" max="7" width="13.140625" style="11" customWidth="1"/>
+    <col min="8" max="8" width="12.42578125" style="12" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" style="12" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28.7109375" style="12" customWidth="1"/>
+    <col min="11" max="11" width="15.28515625" style="12" customWidth="1"/>
+    <col min="12" max="12" width="28.7109375" style="12" customWidth="1"/>
+    <col min="13" max="13" width="15.5703125" style="12" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.7109375" style="12" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6" style="12" bestFit="1" customWidth="1"/>
+    <col min="16" max="21" width="17.7109375" style="12" customWidth="1"/>
+    <col min="22" max="249" width="9.140625" style="5" customWidth="1"/>
+    <col min="250" max="250" width="11.42578125" style="5" customWidth="1"/>
+    <col min="251" max="16384" width="11.42578125" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="3" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" s="3" customFormat="1" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
       <c r="B1" s="2"/>
-      <c r="R1" s="26"/>
-    </row>
-    <row r="2" spans="1:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="U1" s="26"/>
+    </row>
+    <row r="2" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
@@ -1064,7 +1088,7 @@
       </c>
       <c r="G2" s="4"/>
       <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
+      <c r="I2" s="16"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
@@ -1074,8 +1098,11 @@
       <c r="P2" s="4"/>
       <c r="Q2" s="4"/>
       <c r="R2" s="4"/>
-    </row>
-    <row r="3" spans="1:18" s="9" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="S2" s="4"/>
+      <c r="T2" s="4"/>
+      <c r="U2" s="4"/>
+    </row>
+    <row r="3" spans="1:21" s="9" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
         <v>2</v>
       </c>
@@ -1088,52 +1115,61 @@
       <c r="D3" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H3" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="I3" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="J3" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="H3" s="13" t="s">
+      <c r="K3" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="I3" s="8" t="s">
+      <c r="L3" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="J3" s="8" t="s">
+      <c r="M3" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="K3" s="8" t="s">
+      <c r="N3" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="L3" s="8" t="s">
+      <c r="O3" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="M3" s="8" t="s">
+      <c r="P3" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="N3" s="8" t="s">
+      <c r="Q3" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="O3" s="13" t="s">
+      <c r="R3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="P3" s="13" t="s">
+      <c r="S3" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="Q3" s="13" t="s">
+      <c r="T3" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="R3" s="13" t="s">
+      <c r="U3" s="13" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:18" s="36" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:21" s="36" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="30" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="B4" s="31" t="s">
         <v>12</v>
@@ -1144,97 +1180,90 @@
       <c r="D4" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="30" t="s">
+      <c r="E4" s="34" t="s">
+        <v>41</v>
+      </c>
+      <c r="F4" s="34" t="s">
+        <v>43</v>
+      </c>
+      <c r="G4" s="32" t="s">
+        <v>45</v>
+      </c>
+      <c r="H4" s="30" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="34" t="s">
+      <c r="I4" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="34" t="s">
+      <c r="J4" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="35" t="s">
+      <c r="K4" s="35" t="s">
         <v>27</v>
       </c>
-      <c r="I4" s="34" t="s">
+      <c r="L4" s="34" t="s">
         <v>6</v>
       </c>
-      <c r="J4" s="34" t="s">
+      <c r="M4" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="K4" s="34" t="s">
+      <c r="N4" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="L4" s="34" t="s">
+      <c r="O4" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="M4" s="34" t="s">
+      <c r="P4" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="N4" s="34" t="s">
+      <c r="Q4" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="O4" s="35" t="s">
+      <c r="R4" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="P4" s="35" t="s">
+      <c r="S4" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="Q4" s="35" t="s">
+      <c r="T4" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="R4" s="32" t="s">
+      <c r="U4" s="32" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="19"/>
       <c r="B5" s="17"/>
       <c r="C5" s="18"/>
       <c r="D5" s="37"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20"/>
-      <c r="H5" s="22"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="38"/>
+      <c r="H5" s="19"/>
       <c r="I5" s="20"/>
-      <c r="J5" s="21"/>
-      <c r="K5" s="20"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="22"/>
       <c r="L5" s="20"/>
-      <c r="M5" s="20"/>
+      <c r="M5" s="21"/>
       <c r="N5" s="20"/>
-      <c r="O5" s="22"/>
-      <c r="P5" s="22"/>
-      <c r="Q5" s="22"/>
-      <c r="R5" s="23"/>
+      <c r="O5" s="20"/>
+      <c r="P5" s="20"/>
+      <c r="Q5" s="20"/>
+      <c r="R5" s="22"/>
+      <c r="S5" s="22"/>
+      <c r="T5" s="22"/>
+      <c r="U5" s="23"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A5:R9999">
-    <cfRule type="expression" dxfId="1" priority="1">
+  <conditionalFormatting sqref="A5:U9999">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>$B5&lt;&gt;$B4</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation type="date" showInputMessage="1" showErrorMessage="1" sqref="B5:C5" xr:uid="{00000000-0002-0000-0000-000000000000}">
-      <formula1>44927</formula1>
-      <formula2>73050</formula2>
-    </dataValidation>
-    <dataValidation showInputMessage="1" showErrorMessage="1" sqref="D5" xr:uid="{258EF21F-5EC9-4E4F-BCFF-49CA1E9B89AD}"/>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <drawing r:id="rId2"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F37FF43C-AE5E-440A-BDD4-C4D5ADF8CD8D}">
-          <x14:formula1>
-            <xm:f>Rooms!$B$3:$B$9999</xm:f>
-          </x14:formula1>
-          <xm:sqref>A5</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
 </worksheet>
 </file>
 
@@ -1431,4 +1460,44 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12030276-A529-49DE-962D-5EC1ADD71A7E}">
+  <sheetPr>
+    <tabColor theme="0" tint="-0.499984740745262"/>
+  </sheetPr>
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="229" width="9.140625" style="5" customWidth="1"/>
+    <col min="230" max="230" width="11.42578125" style="5" customWidth="1"/>
+    <col min="231" max="16384" width="11.42578125" style="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" s="9" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="27" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" s="10" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A2" s="24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="29" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="29" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
 </file>
</xml_diff>